<commit_message>
Enhance WLS findings statement workflows
</commit_message>
<xml_diff>
--- a/wls_program/docs/wildlife_parsing_codex_lookup.xlsx
+++ b/wls_program/docs/wildlife_parsing_codex_lookup.xlsx
@@ -10,6 +10,7 @@
     <sheet name="RecognitionKeywords" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="RecognitionRegex" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Skips" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="FindingSpecies" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -415,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D282"/>
+  <dimension ref="A1:D286"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4652,6 +4653,86 @@
       <c r="C282" t="inlineStr">
         <is>
           <t>Snowshoe Hare Tracks</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="n">
+        <v>1</v>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>live rabbit</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>Rabbit Sighting</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Exact alias</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="n">
+        <v>1</v>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>wood pecker feeding cavity</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>Pileated Woodpecker Feeding Cavity</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Spelling alias</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="n">
+        <v>1</v>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>moose poop</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>Moose Scat</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Exact alias</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="n">
+        <v>1</v>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>moose</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>Moose Sighting</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Exact alias</t>
         </is>
       </c>
     </row>
@@ -6895,4 +6976,1495 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C89"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>StandardDescription</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>WildlifeGroup</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Abandoned / Inactive Bird Nest</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>BIRDS</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Shed Antler (Moose)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Woodpecker Heard (Audible)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>BIRDS</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Beaver Dam</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Beaver Lodge</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Buck Brushing</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Needs prompt</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Buck Rubbing</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Needs prompt</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Ungulate Scrape</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Shed Antler (Deer)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Deer Tracks</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Woodpecker Cavity Tree</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>BIRDS</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Chicken Scat / Droppings</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>BIRDS</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Coyote Scat</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Coyote Tracks</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Deer Bedding Site</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Deer Scat</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Deer Trail</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Dog Scat</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Dog Tracks</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Fox Tracks</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Moose Tracks</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Grouse Bed</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>BIRDS</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Snowshoe Hare Tracks</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Snowshoe Hare Trail</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Moose Bedding Site</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Moose Scat</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Moose Urine Sign</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Moose Trail</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Snowshoe Hare Scat</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Woodpecker Feeding / Foraging Sign</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>BIRDS</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Wolf Tracks</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Woodpecker Sighting</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>BIRDS</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Animal Remains (Species Unconfirmed)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Needs prompt</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Squirrel Sighting</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Bear Scat</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Possible Bear Tracks</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Beaver Chew</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Chicken Eggshells</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>BIRDS</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Small Mammal Tracks (Unidentified)</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Inactive / Possible Den</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Needs prompt</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Elk Scat</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Elk Tracks</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Elk Trail</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Grouse Sighting</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>BIRDS</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Moose Browse / Feeding Sign</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Owl/Raptor Feeding Sign on Remains</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>BIRDS</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Bird Feather (Unidentified)</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>BIRDS</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Canid Scat (Coyote/Dog)</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Canid Tracks (Coyote/Dog)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Squirrel Drey (Nest)</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>BIRDS</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Squirrel Feeding Sign</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Ungulate Tracks</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Ungulate Rub</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Ungulate Trail</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Woodpecker (Sighting)</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>BIRDS</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Mouse Sighting</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Needs prompt</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Large Game Tracks</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Medium Game Tracks</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Small Game Tracks</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Small Game Trail</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Snowshoe Hare Sighting</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Unidentified Wildlife Sighting</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr"/>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Needs prompt</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Bird Sighting (Unidentified)</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>BIRDS</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Game Tracks</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Game Trail</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Animal Foot Traffic / Active Path</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Needs prompt</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Scat / Droppings (Unidentified)</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Unidentified Wildlife Tracks</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Chicken Sighting</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>BIRDS</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Hair / Fur (Unidentified)</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr"/>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Needs prompt</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Tracks (Unidentified)</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Trail (Unidentified)</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Snowshoe Hare burrow</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Snowshoe Hare Feeding</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Rabbit Sighting</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Pileated Woodpecker Feeding Cavity</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>BIRDS</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Moose Sighting</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Moose Hair / Fur</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Bedding Site (Unidentified)</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Grouse (Mentioned)</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>BIRDS</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Woodpecker (Mentioned)</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>BIRDS</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Tracks Along Cleared Path</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Shed Antler (Unidentified)</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Moose Browsing Activity</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>[Keep Original]</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr"/>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Needs prompt</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Small Rodent Sighting</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Squirrel Tracks</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Beaver Den</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>MAMMALS</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Seeded wildlife group</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>